<commit_message>
chore: clean up website folder + update proof image paths to site subfolders
- Removed: generate_pricing_guide.py, website_service_pricing_guide.pdf, Background/, Ads/capture_proof.py, Ads/ig_logo_export.html, Ads/Proof/gallery.html
- proof.html image paths updated to Ads/Proof/FJMedia.ca/ subfolder structure

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lead Tracker/FJMedia_Lead_Tracker.xlsx
+++ b/Lead Tracker/FJMedia_Lead_Tracker.xlsx
@@ -468,10 +468,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
@@ -480,12 +480,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -536,31 +531,6 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Has Website</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Followers</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Hook</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>DM Sent</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>DM Response</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -594,7 +564,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -603,26 +573,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>341</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>Solid portfolio — bathrooms, basements, commercial builds. Actively hiring so they're growing.</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>B2C pitch angle. Only Facebook in bio.</t>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>No website. Solid portfolio — bathrooms, basements, commercial. Growing (hiring). B2C pitch angle.</t>
         </is>
       </c>
     </row>
@@ -645,7 +598,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>WPG Explore</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -655,7 +608,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr"/>
@@ -664,18 +617,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr"/>
-      <c r="L3" s="5" t="inlineStr"/>
-      <c r="M3" s="4" t="inlineStr"/>
-      <c r="N3" s="4" t="inlineStr"/>
-      <c r="O3" s="5" t="inlineStr">
-        <is>
-          <t>Found via WPG Explore feature.</t>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>No website. Found via WPG Explore.</t>
         </is>
       </c>
     </row>
@@ -708,7 +652,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -717,53 +661,32 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>257</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>Ribbon bouquets, custom orders, consistent product content. Really unique niche.</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>DM to order only. No booking page anywhere.</t>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>No website. Ribbon bouquets, custom orders via DM. Winnipeg-based. 257 followers, consistent content.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Anna</t>
-        </is>
-      </c>
+      <c r="A5" s="4" t="inlineStr"/>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Ms. Groomer</t>
+          <t>FAYNA Pekarnya</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Pet Grooming</t>
+          <t>Bakery</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>@ms_groomer</t>
+          <t>@fayna__pekarnya</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>WPG Explore</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -773,7 +696,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
@@ -782,109 +705,158 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>86</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Breed-standard grooming, 232 posts, solid before/afters. Invisible online despite real skill.</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>No website, no booking page, no directory listing. IG only confirmed via web search.</t>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>No website (Canva link only). 321 followers. Commercial kitchen, licensed. Winnipeg — Nobside Cafe. Cakes, pastries, custom desserts. Already following.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Bright Cleaning Services</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Cleaning</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>@bri.ghtcleaners</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Sugar + Salt Bakeshoppe</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Bakery</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>@sugarandsaltbakeshoppe</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-04-04</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-04-07</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Get Found / Get Customers</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>620</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Residential + commercial cleaning — Yelp link is their only web presence. Multiple service categories, legit operation.</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Yelp in bio. No personal site. Strong niche for trust-based services — a real site = instant credibility boost.</t>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Has Squarespace site (sugarandsaltbakeshoppe.com) — redesign opportunity. 10.7K followers, 897 Corydon Ave. Sweet tables page has no booking form, no pricing, buried lead times. Pitch: better conversion + online ordering flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Gibson's Goodies</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Bakery / Cookies</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>@gibsons.goodies</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>No website. 362 followers. Self-taught cookie decorator. Email: gibsons.goodies.wpg@gmail.com. DM for orders. Winnipeg-based.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Rochelle</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>For Sweet's Sake</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Bakery / Cookies</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>@forsweetssakewpg</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Linktree only (linktr.ee/forsweetssake). 2,644 followers, 409 posts. 'No DMs — email or form.' Strong content, zero web presence. Perfect full site candidate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Cold,Contacted,Replied,Call Booked,Preview Sent,Approved,Paid,Dead,Revisit Later"</formula1>
+      <formula1>"Cold,Contacted,Replied,Call Booked,Preview Sent,Approved,Paid,Dead"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Instagram,WPG Explore,Referral,Cold DM,Comment,Word of Mouth,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Launch $800,Foundation $1400,Authority $2200,Event Site $300,Linktree $300,Retainer Maintain $150,Retainer Grow $300,TBD"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No,Unknown"</formula1>
+      <formula1>"Get Online $300,Get Found $600,Get Customers $1000,Own the Market $1600,Retainer Maintain $150,Retainer Grow $300,TBD"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>